<commit_message>
Fase 6: servicio comercial
- Certificación anual por ascensor con certificado y avisos a 60, 30 y 15 días
  (referencia Acuerdo 470 de 2011 y NTC 5926-1 en Bogotá; norma local configurable).
- Emergencias 24/7 con tiempo objetivo, seguimiento por estados y reporte por QR sin sesión.
- Cotizaciones de correctivos que el cliente aprueba o rechaza desde su portal.
- Indicadores: disponibilidad, MTBF, tiempo medio de respuesta y cumplimiento del plan.
- Documentos e historial del ascensor, sección Próximamente (IoT y predictivo) y recorrido guiado.
- Hojas Certificaciones, Emergencias y Cotizaciones en la plantilla, con exportación e importación.
- docs/PENDIENTES.md con decisiones abiertas y cómo probar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/plantillas/SIGMA_Plantilla_Datos.xlsx
+++ b/backend/resources/plantillas/SIGMA_Plantilla_Datos.xlsx
@@ -9,12 +9,15 @@
     <sheet sheetId="3" name="Edificios" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Ascensores" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Puertas de piso" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Órdenes de trabajo" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Checklist" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Facturas" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Pagos" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Usuarios" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="Listas" state="hidden" r:id="rId14"/>
+    <sheet sheetId="6" name="Certificaciones" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Órdenes de trabajo" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Checklist" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Emergencias" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Cotizaciones" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Facturas" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Pagos" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Usuarios" state="visible" r:id="rId16"/>
+    <sheet sheetId="14" name="Listas" state="hidden" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -29,6 +32,197 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
+          <t>Lo asigna SIGMA (CT-AAAA-00001). Déjelo vacío para crear una cotización.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Código del ascensor (hoja Ascensores). El cliente sale del edificio.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Nombre corto del correctivo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t>Alcance, repuestos y condiciones.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Valor del trabajo sin IVA.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Porcentaje de IVA. Si lo deja vacío, se usa el de la configuración.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Último día para aprobarla. Si la deja vacía, 30 días.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Lo calcula SIGMA.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <t>Esperando respuesta, Aprobada, Rechazada o Vencida.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Código del cliente (hoja Clientes).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Número único de la factura, por ejemplo FV-2210.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>Descripción del cobro.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Fecha de la factura.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. No puede ser anterior a la emisión.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Valor total de la factura.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Lo calcula SIGMA con los pagos registrados.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Pendiente, Abono o Pagada. Lo calcula SIGMA.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Código del cliente que paga.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Número de la factura a la que se aplica el pago.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. No puede superar el saldo de la factura.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Fecha del pago. No puede ser futura.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Transferencia, Consignación, Cheque o Efectivo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Número de la transacción o del recibo. No se puede repetir en la misma factura.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
           <t>Obligatorio. Nombre completo.</t>
         </r>
       </text>
@@ -478,77 +672,63 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Lo asigna SIGMA (OT-AAAA-00001). Déjelo vacío para crear una orden nueva.</t>
+          <t>Obligatorio. Código del ascensor (hoja Ascensores).</t>
         </r>
       </text>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Código del ascensor (hoja Ascensores).</t>
+          <t>Obligatorio. Organismo acreditado por ONAC que hizo la revisión.</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Mantenimiento preventivo, mantenimiento correctivo o inspección.</t>
+          <t>Número que aparece en el certificado.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Baja, Media, Alta o Crítica. Si la deja vacía, queda Media.</t>
+          <t>Norma técnica aplicada. Si la deja vacía, queda NTC 5926-1.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Técnico asignado. Debe estar disponible y sin otra orden en ese horario.</t>
+          <t>Obligatorio. Día de la revisión. No puede ser futura.</t>
         </r>
       </text>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Fecha programada. No puede ser anterior a hoy.</t>
+          <t>Obligatorio. Posterior a la inspección; normalmente un año después.</t>
         </r>
       </text>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Hora programada (24 horas).</t>
+          <t>Obligatorio. Conforme, Conforme con observaciones o No conforme.</t>
         </r>
       </text>
     </comment>
     <comment ref="H1" authorId="0">
       <text>
         <r>
-          <t>Hora estimada de fin. Define la duración (entre 15 minutos y 12 horas).</t>
+          <t>No conformidades o recomendaciones del organismo.</t>
         </r>
       </text>
     </comment>
     <comment ref="I1" authorId="0">
       <text>
         <r>
-          <t>Lo asigna SIGMA: las órdenes nuevas quedan programadas o asignadas.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0">
-      <text>
-        <r>
-          <t>Qué se debe hacer o qué falla reporta el cliente.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0">
-      <text>
-        <r>
-          <t>Notas adicionales.</t>
+          <t>Vigente, Por vencer, Vencida o No conforme. Lo calcula SIGMA.</t>
         </r>
       </text>
     </comment>
@@ -565,42 +745,77 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Orden de mantenimiento preventivo en proceso.</t>
+          <t>Lo asigna SIGMA (OT-AAAA-00001). Déjelo vacío para crear una orden nueva.</t>
         </r>
       </text>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Zona del ascensor.</t>
+          <t>Obligatorio. Código del ascensor (hoja Ascensores).</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Código del ítem (CM-01) o su nombre exacto.</t>
+          <t>Obligatorio. Mantenimiento preventivo, mantenimiento correctivo o inspección.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. B (bueno), R (regular) o M (malo).</t>
+          <t>Baja, Media, Alta o Crítica. Si la deja vacía, queda Media.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. INS, EST o N.A.</t>
+          <t>Técnico asignado. Debe estar disponible y sin otra orden en ese horario.</t>
         </r>
       </text>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
         <r>
-          <t>Obligatoria si el resultado es R o M.</t>
+          <t>Obligatorio. Fecha programada. No puede ser anterior a hoy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Obligatorio. Hora programada (24 horas).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Hora estimada de fin. Define la duración (entre 15 minutos y 12 horas).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <t>Lo asigna SIGMA: las órdenes nuevas quedan programadas o asignadas.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <t>Qué se debe hacer o qué falla reporta el cliente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <t>Notas adicionales.</t>
         </r>
       </text>
     </comment>
@@ -617,56 +832,42 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Código del cliente (hoja Clientes).</t>
+          <t>Obligatorio. Orden de mantenimiento preventivo en proceso.</t>
         </r>
       </text>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Número único de la factura, por ejemplo FV-2210.</t>
+          <t>Obligatorio. Zona del ascensor.</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Descripción del cobro.</t>
+          <t>Obligatorio. Código del ítem (CM-01) o su nombre exacto.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Fecha de la factura.</t>
+          <t>Obligatorio. B (bueno), R (regular) o M (malo).</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. No puede ser anterior a la emisión.</t>
+          <t>Obligatorio. INS, EST o N.A.</t>
         </r>
       </text>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Valor total de la factura.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0">
-      <text>
-        <r>
-          <t>Lo calcula SIGMA con los pagos registrados.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <t>Pendiente, Abono o Pagada. Lo calcula SIGMA.</t>
+          <t>Obligatoria si el resultado es R o M.</t>
         </r>
       </text>
     </comment>
@@ -683,42 +884,98 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Código del cliente que paga.</t>
+          <t>Lo asigna SIGMA (EM-AAAA-00001). Déjelo vacío para registrar una emergencia pasada.</t>
         </r>
       </text>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Número de la factura a la que se aplica el pago.</t>
+          <t>Obligatorio. Código del ascensor (hoja Ascensores).</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. No puede superar el saldo de la factura.</t>
+          <t>Obligatorio. Personas atrapadas, ascensor detenido o con falla, ruido o movimiento anormal, u otro.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Fecha del pago. No puede ser futura.</t>
+          <t>Obligatorio. Día en que se reportó. No puede ser futura.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Transferencia, Consignación, Cheque o Efectivo.</t>
+          <t>Obligatorio. Hora del reporte (24 horas).</t>
         </r>
       </text>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
         <r>
-          <t>Obligatorio. Número de la transacción o del recibo. No se puede repetir en la misma factura.</t>
+          <t>Nombre de quien avisó (portería, residente, administrador).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Teléfono de contacto.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Qué pasó.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <t>Técnico que atendió.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <t>Hora en que llegó el técnico, el mismo día del reporte. Sirve para el tiempo de respuesta.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <t>Día en que quedó resuelta. Si la deja vacía, la emergencia queda abierta.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <t>Hora en que quedó resuelta.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <r>
+          <t>Qué se hizo. Obligatoria si escribe la fecha de solución.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <t>Lo calcula SIGMA.</t>
         </r>
       </text>
     </comment>
@@ -727,7 +984,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="233">
   <si>
     <t>SIGMA · Plantilla de carga de datos</t>
   </si>
@@ -750,13 +1007,13 @@
     <t>4. La fila 2 de cada hoja es un ejemplo: su primer valor empieza por EJEMPLO y SIGMA la ignora al importar. Puede borrarla o dejarla.</t>
   </si>
   <si>
-    <t>5. Los códigos relacionan las hojas: el código del cliente une Clientes, Edificios, Ascensores, Facturas y Pagos; el código del ascensor une Ascensores, Puertas de piso y Órdenes de trabajo.</t>
+    <t>5. Los códigos relacionan las hojas: el código del cliente une Clientes, Edificios, Ascensores, Facturas y Pagos; el código del ascensor une Ascensores, Puertas de piso, Certificaciones, Órdenes de trabajo, Emergencias y Cotizaciones.</t>
   </si>
   <si>
     <t>Orden de carga</t>
   </si>
   <si>
-    <t>Clientes → Edificios → Ascensores → Puertas de piso → Órdenes de trabajo → Checklist → Facturas → Pagos → Usuarios.</t>
+    <t>Clientes → Edificios → Ascensores → Puertas de piso → Certificaciones → Órdenes de trabajo → Checklist → Emergencias → Cotizaciones → Facturas → Pagos → Usuarios.</t>
   </si>
   <si>
     <t>Puede subir todas las hojas en un solo archivo: SIGMA las procesa en ese orden.</t>
@@ -783,12 +1040,15 @@
     <t>Si un código ya existe en SIGMA, la fila actualiza ese registro en lugar de crear otro. Exporte, corrija en Excel y vuelva a importar sin perder información.</t>
   </si>
   <si>
-    <t>Las órdenes de trabajo, facturas y pagos que ya existen no se modifican desde Excel; se informan como existentes.</t>
+    <t>Las órdenes de trabajo, emergencias, cotizaciones, certificaciones, facturas y pagos que ya existen no se modifican desde Excel; se informan como existentes.</t>
   </si>
   <si>
     <t>Al importar ascensores, SIGMA crea una puerta de piso por cada parada. La hoja Puertas de piso sirve para indicar su tipo y estado.</t>
   </si>
   <si>
+    <t>Certificación anual: en Bogotá la revisión general anual la exige el Acuerdo 470 de 2011 y se hace con la NTC 5926-1 por un organismo acreditado por ONAC. En otras ciudades registre la norma que aplique.</t>
+  </si>
+  <si>
     <t>Código *</t>
   </si>
   <si>
@@ -1002,6 +1262,36 @@
     <t>Cierre lento, roce en la zapata.</t>
   </si>
   <si>
+    <t>Organismo de inspección *</t>
+  </si>
+  <si>
+    <t>Número del certificado</t>
+  </si>
+  <si>
+    <t>Norma</t>
+  </si>
+  <si>
+    <t>Fecha de inspección *</t>
+  </si>
+  <si>
+    <t>Fecha de vencimiento *</t>
+  </si>
+  <si>
+    <t>Resultado *</t>
+  </si>
+  <si>
+    <t>Inspecciones Andinas S.A.S.</t>
+  </si>
+  <si>
+    <t>RA-2026-118</t>
+  </si>
+  <si>
+    <t>NTC 5926-1</t>
+  </si>
+  <si>
+    <t>Conforme</t>
+  </si>
+  <si>
     <t>Número</t>
   </si>
   <si>
@@ -1041,9 +1331,6 @@
     <t>Ítem *</t>
   </si>
   <si>
-    <t>Resultado *</t>
-  </si>
-  <si>
     <t>EJEMPLO-OT-2026-00004</t>
   </si>
   <si>
@@ -1059,6 +1346,69 @@
     <t>INS</t>
   </si>
   <si>
+    <t>Fecha del reporte *</t>
+  </si>
+  <si>
+    <t>Hora del reporte *</t>
+  </si>
+  <si>
+    <t>Quién reportó</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Hora de llegada</t>
+  </si>
+  <si>
+    <t>Fecha de solución</t>
+  </si>
+  <si>
+    <t>Hora de solución</t>
+  </si>
+  <si>
+    <t>Solución</t>
+  </si>
+  <si>
+    <t>Personas atrapadas</t>
+  </si>
+  <si>
+    <t>Portería Torre A</t>
+  </si>
+  <si>
+    <t>601 555 1234</t>
+  </si>
+  <si>
+    <t>Cabina detenida entre los pisos 3 y 4.</t>
+  </si>
+  <si>
+    <t>Rescate y ajuste del freno.</t>
+  </si>
+  <si>
+    <t>Trabajo cotizado *</t>
+  </si>
+  <si>
+    <t>Detalle</t>
+  </si>
+  <si>
+    <t>Valor antes de IVA (COP) *</t>
+  </si>
+  <si>
+    <t>IVA (%)</t>
+  </si>
+  <si>
+    <t>Vigente hasta</t>
+  </si>
+  <si>
+    <t>Total (COP)</t>
+  </si>
+  <si>
+    <t>Cambio de amortiguadores del foso</t>
+  </si>
+  <si>
+    <t>Incluye dos amortiguadores hidráulicos y mano de obra.</t>
+  </si>
+  <si>
     <t>Factura *</t>
   </si>
   <si>
@@ -1068,9 +1418,6 @@
     <t>Fecha de emisión *</t>
   </si>
   <si>
-    <t>Fecha de vencimiento *</t>
-  </si>
-  <si>
     <t>Valor (COP) *</t>
   </si>
   <si>
@@ -1173,6 +1520,12 @@
     <t>planes</t>
   </si>
   <si>
+    <t>tiposEmergencia</t>
+  </si>
+  <si>
+    <t>resultadosCertificacion</t>
+  </si>
+  <si>
     <t>CC</t>
   </si>
   <si>
@@ -1233,6 +1586,12 @@
     <t>Coordinador</t>
   </si>
   <si>
+    <t>Ascensor detenido o con falla</t>
+  </si>
+  <si>
+    <t>Conforme con observaciones</t>
+  </si>
+  <si>
     <t>TI</t>
   </si>
   <si>
@@ -1266,6 +1625,12 @@
     <t>Cheque</t>
   </si>
   <si>
+    <t>Ruido o movimiento anormal</t>
+  </si>
+  <si>
+    <t>No conforme</t>
+  </si>
+  <si>
     <t>PA</t>
   </si>
   <si>
@@ -1288,6 +1653,9 @@
   </si>
   <si>
     <t>Contador</t>
+  </si>
+  <si>
+    <t>Otro</t>
   </si>
   <si>
     <t>Mitsubishi</t>
@@ -1810,7 +2178,7 @@
   <sheetPr>
     <tabColor rgb="FF4E29AA"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
@@ -1936,6 +2304,16 @@
         <v>19</v>
       </c>
     </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1943,6 +2321,261 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF22124A"/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="18" style="5" customWidth="1"/>
+    <col min="6" max="6" width="10" style="16" customWidth="1"/>
+    <col min="7" max="7" width="14" style="4" customWidth="1"/>
+    <col min="8" max="8" width="16" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" s="12">
+        <v>2000000</v>
+      </c>
+      <c r="F2" s="18">
+        <v>19</v>
+      </c>
+      <c r="G2" s="11">
+        <v>46356</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
+  <dataValidations count="4">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor antes de IVA (COP)" error="Escriba el valor en pesos, sin decimales." sqref="E2:E2000">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="IVA (%)" error="Escriba un número entre 0 y 100." sqref="F2:F2000">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Vigente hasta" error="Escriba una fecha válida (día/mes/año)." sqref="G2:G2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Total (COP)" error="Escriba el valor en pesos, sin decimales." sqref="H2:H2000">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF22124A"/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="5" width="14" style="4" customWidth="1"/>
+    <col min="6" max="7" width="16" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="11">
+        <v>46300</v>
+      </c>
+      <c r="E2" s="11">
+        <v>46315</v>
+      </c>
+      <c r="F2" s="12">
+        <v>850000</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1"/>
+  <dataValidations count="4">
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de emisión" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de vencimiento" error="Escriba una fecha válida (día/mes/año)." sqref="E2:E2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor (COP)" error="Escriba el valor en pesos, sin decimales." sqref="F2:F2000">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Saldo (COP)" error="Escriba el valor en pesos, sin decimales." sqref="G2:G2000">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF22124A"/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13" style="4" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="12">
+        <v>850000</v>
+      </c>
+      <c r="D2" s="11">
+        <v>46313</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="3">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor (COP)" error="Escriba el valor en pesos, sin decimales." sqref="C2:C2000">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Medio de pago" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
+      <formula1>Listas!$P$2:$P$500</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF22124A"/>
@@ -1959,36 +2592,36 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2010,289 +2643,316 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="19" width="28" customWidth="1"/>
+    <col min="1" max="21" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>136</v>
+        <v>166</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="K1" s="23" t="s">
-        <v>139</v>
+        <v>169</v>
       </c>
       <c r="L1" s="23" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="M1" s="23" t="s">
-        <v>141</v>
+        <v>171</v>
       </c>
       <c r="N1" s="23" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="O1" s="23" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="P1" s="23" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="Q1" s="23" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="R1" s="23" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
       <c r="S1" s="23" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+      <c r="T1" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="U1" s="23" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="F2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J2" t="s">
+        <v>182</v>
+      </c>
+      <c r="K2" t="s">
+        <v>183</v>
+      </c>
+      <c r="L2" t="s">
+        <v>184</v>
+      </c>
+      <c r="M2" t="s">
+        <v>116</v>
+      </c>
+      <c r="N2" t="s">
+        <v>118</v>
+      </c>
+      <c r="O2" t="s">
+        <v>119</v>
+      </c>
+      <c r="P2" t="s">
         <v>150</v>
       </c>
-      <c r="K2" t="s">
-        <v>151</v>
-      </c>
-      <c r="L2" t="s">
-        <v>152</v>
-      </c>
-      <c r="M2" t="s">
-        <v>106</v>
-      </c>
-      <c r="N2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
+        <v>185</v>
+      </c>
+      <c r="T2" t="s">
+        <v>128</v>
+      </c>
+      <c r="U2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G3" t="s">
+        <v>191</v>
+      </c>
+      <c r="H3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K3" t="s">
         <v>109</v>
       </c>
-      <c r="P2" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D3" t="s">
-        <v>157</v>
-      </c>
-      <c r="E3" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" t="s">
-        <v>159</v>
-      </c>
-      <c r="H3" t="s">
-        <v>160</v>
-      </c>
-      <c r="I3" t="s">
-        <v>161</v>
-      </c>
-      <c r="J3" t="s">
-        <v>89</v>
-      </c>
-      <c r="K3" t="s">
-        <v>98</v>
-      </c>
       <c r="L3" t="s">
-        <v>162</v>
+        <v>194</v>
       </c>
       <c r="M3" t="s">
-        <v>163</v>
+        <v>195</v>
       </c>
       <c r="N3" t="s">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="O3" t="s">
-        <v>165</v>
+        <v>197</v>
       </c>
       <c r="P3" t="s">
-        <v>166</v>
+        <v>198</v>
       </c>
       <c r="Q3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+      <c r="T3" t="s">
+        <v>200</v>
+      </c>
+      <c r="U3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>168</v>
+        <v>202</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E4" t="s">
-        <v>170</v>
+        <v>204</v>
       </c>
       <c r="F4" t="s">
-        <v>171</v>
+        <v>205</v>
       </c>
       <c r="G4" t="s">
-        <v>172</v>
+        <v>206</v>
       </c>
       <c r="H4" t="s">
-        <v>156</v>
+        <v>188</v>
       </c>
       <c r="J4" t="s">
-        <v>173</v>
+        <v>207</v>
       </c>
       <c r="K4" t="s">
-        <v>174</v>
+        <v>208</v>
       </c>
       <c r="L4" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="M4" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="N4" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
       <c r="O4" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="P4" t="s">
-        <v>178</v>
+        <v>212</v>
       </c>
       <c r="Q4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+      <c r="T4" t="s">
+        <v>213</v>
+      </c>
+      <c r="U4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>179</v>
+        <v>215</v>
       </c>
       <c r="E5" t="s">
-        <v>180</v>
+        <v>216</v>
       </c>
       <c r="G5" t="s">
-        <v>181</v>
+        <v>217</v>
       </c>
       <c r="J5" t="s">
-        <v>182</v>
+        <v>218</v>
       </c>
       <c r="L5" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
       <c r="M5" t="s">
-        <v>184</v>
+        <v>220</v>
       </c>
       <c r="P5" t="s">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="Q5" t="s">
-        <v>186</v>
+        <v>222</v>
+      </c>
+      <c r="T5" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
-        <v>187</v>
+        <v>224</v>
       </c>
       <c r="M6" t="s">
-        <v>188</v>
+        <v>225</v>
       </c>
       <c r="Q6" t="s">
-        <v>189</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
-        <v>190</v>
+        <v>227</v>
       </c>
       <c r="M7" t="s">
-        <v>191</v>
+        <v>228</v>
       </c>
       <c r="Q7" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
-        <v>192</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>193</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>194</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>195</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2325,73 +2985,73 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="11">
@@ -2404,7 +3064,7 @@
         <v>18000000</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2462,70 +3122,70 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G2" s="15">
         <v>18</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2584,96 +3244,96 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R1" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G2" s="15">
         <v>2018</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I2" s="15">
         <v>630</v>
@@ -2688,13 +3348,13 @@
         <v>7</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="P2" s="15">
         <v>1</v>
@@ -2708,7 +3368,7 @@
         <v>380000</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2787,36 +3447,36 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="15">
         <v>6</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2840,6 +3500,97 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF22124A"/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="6" width="14" style="4" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="11">
+        <v>46091</v>
+      </c>
+      <c r="F2" s="11">
+        <v>46456</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
+  <dataValidations count="3">
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de inspección" error="Escriba una fecha válida (día/mes/año)." sqref="E2:E2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de vencimiento" error="Escriba una fecha válida (día/mes/año)." sqref="F2:F2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Resultado" error="Elija un valor de la lista desplegable." sqref="G2:G2000">
+      <formula1>Listas!$U$2:$U$500</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF22124A"/>
@@ -2861,49 +3612,49 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="11">
@@ -2917,7 +3668,7 @@
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="10" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2951,7 +3702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF22124A"/>
@@ -2969,39 +3720,39 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3015,92 +3766,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
       <formula1>Listas!$O$2:$O$500</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FF22124A"/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="5" width="14" style="4" customWidth="1"/>
-    <col min="6" max="7" width="16" style="5" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G1" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="D2" s="11">
-        <v>46300</v>
-      </c>
-      <c r="E2" s="11">
-        <v>46315</v>
-      </c>
-      <c r="F2" s="12">
-        <v>850000</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H1"/>
-  <dataValidations count="4">
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de emisión" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
-      <formula1>21916</formula1>
-      <formula2>73415</formula2>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de vencimiento" error="Escriba una fecha válida (día/mes/año)." sqref="E2:E2000">
-      <formula1>21916</formula1>
-      <formula2>73415</formula2>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor (COP)" error="Escriba el valor en pesos, sin decimales." sqref="F2:F2000">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Saldo (COP)" error="Escriba el valor en pesos, sin decimales." sqref="G2:G2000">
-      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3114,69 +3779,134 @@
   <sheetPr>
     <tabColor rgb="FF22124A"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="16" style="5" customWidth="1"/>
-    <col min="4" max="4" width="13" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="14" style="4" customWidth="1"/>
+    <col min="5" max="5" width="12" style="19" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="12" style="19" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="12" style="19" customWidth="1"/>
+    <col min="13" max="13" width="34" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>43</v>
+    <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>102</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>114</v>
+        <v>85</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>46</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>121</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J1" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="L1" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="N1" s="7" t="s">
         <v>34</v>
       </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C2" s="12">
-        <v>850000</v>
+        <v>77</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>128</v>
       </c>
       <c r="D2" s="11">
-        <v>46313</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>120</v>
+        <v>46307</v>
+      </c>
+      <c r="E2" s="21">
+        <v>0.8194444444444444</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>121</v>
+        <v>129</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="I2" s="10"/>
+      <c r="J2" s="21">
+        <v>0.8368055555555556</v>
+      </c>
+      <c r="K2" s="11">
+        <v>46307</v>
+      </c>
+      <c r="L2" s="21">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
-  <dataValidations count="3">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor (COP)" error="Escriba el valor en pesos, sin decimales." sqref="C2:C2000">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
+  <autoFilter ref="A1:N1"/>
+  <dataValidations count="7">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="C2:C2000">
+      <formula1>Listas!$T$2:$T$500</formula1>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha del reporte" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
       <formula1>21916</formula1>
       <formula2>73415</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Medio de pago" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
-      <formula1>Listas!$P$2:$P$500</formula1>
+    <dataValidation type="time" allowBlank="1" showErrorMessage="1" errorTitle="Hora del reporte" error="Escriba una hora en formato 24 horas (07:30)." sqref="E2:E2000">
+      <formula1>0</formula1>
+      <formula2>0.99999</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Técnico" error="Elija un valor de la lista desplegable." sqref="I2:I2000">
+      <formula1>Listas!$R$2:$R$500</formula1>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showErrorMessage="1" errorTitle="Hora de llegada" error="Escriba una hora en formato 24 horas (07:30)." sqref="J2:J2000">
+      <formula1>0</formula1>
+      <formula2>0.99999</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha de solución" error="Escriba una fecha válida (día/mes/año)." sqref="K2:K2000">
+      <formula1>21916</formula1>
+      <formula2>73415</formula2>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showErrorMessage="1" errorTitle="Hora de solución" error="Escriba una hora en formato 24 horas (07:30)." sqref="L2:L2000">
+      <formula1>0</formula1>
+      <formula2>0.99999</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Tipos de ascensor, aviso al revisar Excel y ajustes del panel en el celular
- Tipo de ascensor por uso (pasajeros, carga, camillero, panorámico, vehicular, plataforma,
  montaplatos): ficha, formulario, filtro y columna en la lista, plantilla de Excel y app.
- Importar: panel "Revisando…" con barra de progreso y notificación que cambia al resultado.
- Celular: el menú lateral se cierra al tocar fuera (o con Esc); botones del pie de los modales
  apilados; errores de importación como fichas.
- Validación: "posterior o igual a hoy" en lugar de "today".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/plantillas/SIGMA_Plantilla_Datos.xlsx
+++ b/backend/resources/plantillas/SIGMA_Plantilla_Datos.xlsx
@@ -547,67 +547,74 @@
     <comment ref="M1" authorId="0">
       <text>
         <r>
+          <t>Uso del ascensor: pasajeros, carga, camillero, panorámico, vehicular, plataforma o montaplatos.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
           <t>Elija de la lista o escriba el tipo de accionamiento.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <t>Controlador o tablero de maniobra.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <t>Elija de la lista o escriba el tipo de la puerta de cabina.</t>
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
+    <comment ref="Q1" authorId="0">
       <text>
         <r>
           <t>Cada cuántos meses se hace el mantenimiento preventivo (1 a 6). Si la llena, también llene la fecha del primer mantenimiento.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="R1" authorId="0">
       <text>
         <r>
           <t>Plan de mantenimiento. Si lo deja vacío, se usa el primer plan activo con esa periodicidad.</t>
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <t>Fecha desde la que se programan las visitas.</t>
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <t>Técnico de referencia del ascensor (debe estar registrado en SIGMA).</t>
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <t>Precio pactado por visita. Si lo deja vacío, se usa el precio del plan.</t>
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0">
+    <comment ref="V1" authorId="0">
       <text>
         <r>
           <t>Activo, En mantenimiento o Inactivo.</t>
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0">
+    <comment ref="W1" authorId="0">
       <text>
         <r>
           <t>Notas generales del equipo.</t>
@@ -984,7 +991,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="242">
   <si>
     <t>SIGMA · Plantilla de carga de datos</t>
   </si>
@@ -1190,6 +1197,9 @@
     <t>Paradas *</t>
   </si>
   <si>
+    <t>Tipo de ascensor</t>
+  </si>
+  <si>
     <t>Accionamiento</t>
   </si>
   <si>
@@ -1232,6 +1242,9 @@
     <t>SN-4471</t>
   </si>
   <si>
+    <t>Pasajeros</t>
+  </si>
+  <si>
     <t>Eléctrico de tracción</t>
   </si>
   <si>
@@ -1478,6 +1491,9 @@
     <t>marcas</t>
   </si>
   <si>
+    <t>tiposAscensor</t>
+  </si>
+  <si>
     <t>accionamientos</t>
   </si>
   <si>
@@ -1556,6 +1572,9 @@
     <t>Institucional</t>
   </si>
   <si>
+    <t>Carga (montacargas)</t>
+  </si>
+  <si>
     <t>Eléctrico sin cuarto de máquinas (MRL)</t>
   </si>
   <si>
@@ -1601,6 +1620,9 @@
     <t>Kone</t>
   </si>
   <si>
+    <t>Camillero (hospitalario)</t>
+  </si>
+  <si>
     <t>Hidráulico</t>
   </si>
   <si>
@@ -1637,6 +1659,9 @@
     <t>TK Elevator</t>
   </si>
   <si>
+    <t>Panorámico</t>
+  </si>
+  <si>
     <t>Manual de tijera</t>
   </si>
   <si>
@@ -1661,6 +1686,9 @@
     <t>Mitsubishi</t>
   </si>
   <si>
+    <t>Vehicular</t>
+  </si>
+  <si>
     <t>Hueco y recorrido</t>
   </si>
   <si>
@@ -1670,10 +1698,16 @@
     <t>Orona</t>
   </si>
   <si>
+    <t>Plataforma para movilidad reducida</t>
+  </si>
+  <si>
     <t>Foso</t>
   </si>
   <si>
     <t>Hyundai</t>
+  </si>
+  <si>
+    <t>Montaplatos</t>
   </si>
   <si>
     <t>Fujitec</t>
@@ -2341,28 +2375,28 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>34</v>
@@ -2371,13 +2405,13 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E2" s="12">
         <v>2000000</v>
@@ -2434,22 +2468,22 @@
         <v>44</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>34</v>
@@ -2460,10 +2494,10 @@
         <v>35</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D2" s="11">
         <v>46300</v>
@@ -2520,19 +2554,19 @@
         <v>44</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2540,7 +2574,7 @@
         <v>35</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C2" s="12">
         <v>850000</v>
@@ -2549,10 +2583,10 @@
         <v>46313</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2566,7 +2600,7 @@
       <formula2>73415</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Medio de pago" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
-      <formula1>Listas!$P$2:$P$500</formula1>
+      <formula1>Listas!$Q$2:$Q$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2592,30 +2626,30 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>43</v>
@@ -2631,7 +2665,7 @@
       <formula1>ISNUMBER(SEARCH("@",B2))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Rol" error="Elija un valor de la lista desplegable." sqref="C2:C2000">
-      <formula1>Listas!$Q$2:$Q$500</formula1>
+      <formula1>Listas!$R$2:$R$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Estado" error="Elija un valor de la lista desplegable." sqref="D2:D2000">
       <formula1>Listas!$C$2:$C$500</formula1>
@@ -2645,83 +2679,86 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="21" width="28" customWidth="1"/>
+    <col min="1" max="22" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="K1" s="23" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L1" s="23" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="M1" s="23" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="N1" s="23" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="O1" s="23" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P1" s="23" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="Q1" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="R1" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="S1" s="23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="T1" s="23" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="U1" s="23" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+      <c r="V1" s="23" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
         <v>43</v>
@@ -2730,229 +2767,250 @@
         <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G2" t="s">
         <v>84</v>
       </c>
       <c r="H2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I2" t="s">
         <v>43</v>
       </c>
-      <c r="I2" t="s">
-        <v>89</v>
-      </c>
       <c r="J2" t="s">
-        <v>182</v>
+        <v>91</v>
       </c>
       <c r="K2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="M2" t="s">
-        <v>116</v>
+        <v>187</v>
       </c>
       <c r="N2" t="s">
         <v>118</v>
       </c>
       <c r="O2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P2" t="s">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="Q2" t="s">
-        <v>185</v>
-      </c>
-      <c r="T2" t="s">
-        <v>128</v>
+        <v>152</v>
+      </c>
+      <c r="R2" t="s">
+        <v>188</v>
       </c>
       <c r="U2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="V2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H3" t="s">
+        <v>195</v>
+      </c>
+      <c r="I3" t="s">
+        <v>196</v>
+      </c>
+      <c r="J3" t="s">
+        <v>197</v>
+      </c>
+      <c r="K3" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" t="s">
+        <v>111</v>
+      </c>
+      <c r="M3" t="s">
+        <v>198</v>
+      </c>
+      <c r="N3" t="s">
+        <v>199</v>
+      </c>
+      <c r="O3" t="s">
+        <v>200</v>
+      </c>
+      <c r="P3" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>202</v>
+      </c>
+      <c r="R3" t="s">
+        <v>203</v>
+      </c>
+      <c r="U3" t="s">
+        <v>204</v>
+      </c>
+      <c r="V3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" t="s">
+        <v>207</v>
+      </c>
+      <c r="E4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H4" t="s">
+        <v>211</v>
+      </c>
+      <c r="I4" t="s">
         <v>191</v>
       </c>
-      <c r="H3" t="s">
-        <v>192</v>
-      </c>
-      <c r="I3" t="s">
-        <v>193</v>
-      </c>
-      <c r="J3" t="s">
-        <v>90</v>
-      </c>
-      <c r="K3" t="s">
-        <v>109</v>
-      </c>
-      <c r="L3" t="s">
-        <v>194</v>
-      </c>
-      <c r="M3" t="s">
-        <v>195</v>
-      </c>
-      <c r="N3" t="s">
-        <v>196</v>
-      </c>
-      <c r="O3" t="s">
-        <v>197</v>
-      </c>
-      <c r="P3" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>199</v>
-      </c>
-      <c r="T3" t="s">
-        <v>200</v>
-      </c>
-      <c r="U3" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D4" t="s">
-        <v>203</v>
-      </c>
-      <c r="E4" t="s">
-        <v>204</v>
-      </c>
-      <c r="F4" t="s">
-        <v>205</v>
-      </c>
-      <c r="G4" t="s">
-        <v>206</v>
-      </c>
-      <c r="H4" t="s">
-        <v>188</v>
-      </c>
-      <c r="J4" t="s">
-        <v>207</v>
-      </c>
       <c r="K4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="L4" t="s">
-        <v>110</v>
+        <v>213</v>
       </c>
       <c r="M4" t="s">
-        <v>209</v>
+        <v>112</v>
       </c>
       <c r="N4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="O4" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="P4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="Q4" t="s">
-        <v>104</v>
-      </c>
-      <c r="T4" t="s">
-        <v>213</v>
+        <v>217</v>
+      </c>
+      <c r="R4" t="s">
+        <v>106</v>
       </c>
       <c r="U4" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="V4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E5" t="s">
-        <v>216</v>
-      </c>
-      <c r="G5" t="s">
-        <v>217</v>
-      </c>
-      <c r="J5" t="s">
-        <v>218</v>
-      </c>
-      <c r="L5" t="s">
-        <v>219</v>
+        <v>221</v>
+      </c>
+      <c r="F5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H5" t="s">
+        <v>223</v>
+      </c>
+      <c r="K5" t="s">
+        <v>224</v>
       </c>
       <c r="M5" t="s">
-        <v>220</v>
-      </c>
-      <c r="P5" t="s">
-        <v>221</v>
+        <v>225</v>
+      </c>
+      <c r="N5" t="s">
+        <v>226</v>
       </c>
       <c r="Q5" t="s">
-        <v>222</v>
-      </c>
-      <c r="T5" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="6" spans="5:17" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+      <c r="R5" t="s">
+        <v>228</v>
+      </c>
+      <c r="U5" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
-        <v>224</v>
-      </c>
-      <c r="M6" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="7" spans="5:17" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+      <c r="F6" t="s">
+        <v>231</v>
+      </c>
+      <c r="N6" t="s">
+        <v>232</v>
+      </c>
+      <c r="R6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
-        <v>227</v>
-      </c>
-      <c r="M7" t="s">
-        <v>228</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" spans="5:5" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+      <c r="F7" t="s">
+        <v>235</v>
+      </c>
+      <c r="N7" t="s">
+        <v>236</v>
+      </c>
+      <c r="R7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
-        <v>229</v>
+        <v>237</v>
+      </c>
+      <c r="F8" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -3216,7 +3274,7 @@
   <sheetPr>
     <tabColor rgb="FF22124A"/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3230,19 +3288,20 @@
     <col min="10" max="10" width="10" style="13" customWidth="1"/>
     <col min="11" max="11" width="12" style="16" customWidth="1"/>
     <col min="12" max="12" width="10" style="13" customWidth="1"/>
-    <col min="13" max="13" width="26" customWidth="1"/>
-    <col min="14" max="14" width="18" customWidth="1"/>
-    <col min="15" max="15" width="26" customWidth="1"/>
-    <col min="16" max="16" width="13" style="13" customWidth="1"/>
-    <col min="17" max="17" width="24" customWidth="1"/>
-    <col min="18" max="18" width="16" style="4" customWidth="1"/>
-    <col min="19" max="19" width="22" customWidth="1"/>
-    <col min="20" max="20" width="18" style="5" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
-    <col min="22" max="22" width="30" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="14" width="26" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="26" customWidth="1"/>
+    <col min="17" max="17" width="13" style="13" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="16" style="4" customWidth="1"/>
+    <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="18" style="5" customWidth="1"/>
+    <col min="22" max="22" width="16" customWidth="1"/>
+    <col min="23" max="23" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>21</v>
       </c>
@@ -3288,31 +3347,34 @@
       <c r="O1" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="P1" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="V1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="W1" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>35</v>
@@ -3321,19 +3383,19 @@
         <v>54</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="15">
         <v>2018</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I2" s="15">
         <v>630</v>
@@ -3348,32 +3410,35 @@
         <v>7</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="P2" s="15">
+        <v>85</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q2" s="15">
         <v>1</v>
       </c>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="11">
+      <c r="R2" s="10"/>
+      <c r="S2" s="11">
         <v>46329</v>
       </c>
-      <c r="S2" s="10"/>
-      <c r="T2" s="12">
+      <c r="T2" s="10"/>
+      <c r="U2" s="12">
         <v>380000</v>
       </c>
-      <c r="U2" s="10" t="s">
+      <c r="V2" s="10" t="s">
         <v>43</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V1"/>
-  <dataValidations count="14">
+  <autoFilter ref="A1:W1"/>
+  <dataValidations count="15">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="information" errorTitle="Marca" error="El valor no está en la lista. Puede conservarlo si es correcto." sqref="E2:E2000">
       <formula1>Listas!$E$2:$E$500</formula1>
     </dataValidation>
@@ -3397,31 +3462,34 @@
       <formula1>2</formula1>
       <formula2>60</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="information" errorTitle="Accionamiento" error="El valor no está en la lista. Puede conservarlo si es correcto." sqref="M2:M2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo de ascensor" error="Elija un valor de la lista desplegable." sqref="M2:M2000">
       <formula1>Listas!$F$2:$F$500</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="information" errorTitle="Tipo de puerta de cabina" error="El valor no está en la lista. Puede conservarlo si es correcto." sqref="O2:O2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="information" errorTitle="Accionamiento" error="El valor no está en la lista. Puede conservarlo si es correcto." sqref="N2:N2000">
       <formula1>Listas!$G$2:$G$500</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Periodicidad (meses)" error="Escriba un número entero entre 1 y 6." sqref="P2:P2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="information" errorTitle="Tipo de puerta de cabina" error="El valor no está en la lista. Puede conservarlo si es correcto." sqref="P2:P2000">
+      <formula1>Listas!$H$2:$H$500</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Periodicidad (meses)" error="Escriba un número entero entre 1 y 6." sqref="Q2:Q2000">
       <formula1>1</formula1>
       <formula2>6</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Plan" error="Elija un valor de la lista desplegable." sqref="Q2:Q2000">
-      <formula1>Listas!$S$2:$S$500</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha del primer mantenimiento" error="Escriba una fecha válida (día/mes/año)." sqref="R2:R2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Plan" error="Elija un valor de la lista desplegable." sqref="R2:R2000">
+      <formula1>Listas!$T$2:$T$500</formula1>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha del primer mantenimiento" error="Escriba una fecha válida (día/mes/año)." sqref="S2:S2000">
       <formula1>21916</formula1>
       <formula2>73415</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Técnico asignado" error="Elija un valor de la lista desplegable." sqref="S2:S2000">
-      <formula1>Listas!$R$2:$R$500</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor por visita (COP)" error="Escriba el valor en pesos, sin decimales." sqref="T2:T2000">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Técnico asignado" error="Elija un valor de la lista desplegable." sqref="T2:T2000">
+      <formula1>Listas!$S$2:$S$500</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Valor por visita (COP)" error="Escriba el valor en pesos, sin decimales." sqref="U2:U2000">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Estado" error="Elija un valor de la lista desplegable." sqref="U2:U2000">
-      <formula1>Listas!$H$2:$H$500</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Estado" error="Elija un valor de la lista desplegable." sqref="V2:V2000">
+      <formula1>Listas!$I$2:$I$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3447,36 +3515,36 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="15">
         <v>6</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -3487,10 +3555,10 @@
       <formula2>60</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="C2:C2000">
-      <formula1>Listas!$I$2:$I$500</formula1>
+      <formula1>Listas!$J$2:$J$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Estado" error="Elija un valor de la lista desplegable." sqref="D2:D2000">
-      <formula1>Listas!$J$2:$J$500</formula1>
+      <formula1>Listas!$K$2:$K$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3519,28 +3587,28 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>34</v>
@@ -3548,16 +3616,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E2" s="11">
         <v>46091</v>
@@ -3566,7 +3634,7 @@
         <v>46456</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -3581,7 +3649,7 @@
       <formula2>73415</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Resultado" error="Elija un valor de la lista desplegable." sqref="G2:G2000">
-      <formula1>Listas!$U$2:$U$500</formula1>
+      <formula1>Listas!$V$2:$V$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3612,49 +3680,49 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>34</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="11">
@@ -3668,20 +3736,20 @@
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="C2:C2000">
-      <formula1>Listas!$K$2:$K$500</formula1>
+      <formula1>Listas!$L$2:$L$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Prioridad" error="Elija un valor de la lista desplegable." sqref="D2:D2000">
-      <formula1>Listas!$L$2:$L$500</formula1>
+      <formula1>Listas!$M$2:$M$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Técnico" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
-      <formula1>Listas!$R$2:$R$500</formula1>
+      <formula1>Listas!$S$2:$S$500</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha" error="Escriba una fecha válida (día/mes/año)." sqref="F2:F2000">
       <formula1>21916</formula1>
@@ -3720,52 +3788,52 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>46</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Zona" error="Elija un valor de la lista desplegable." sqref="B2:B2000">
-      <formula1>Listas!$M$2:$M$500</formula1>
+      <formula1>Listas!$N$2:$N$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Resultado" error="Elija un valor de la lista desplegable." sqref="D2:D2000">
-      <formula1>Listas!$N$2:$N$500</formula1>
+      <formula1>Listas!$O$2:$O$500</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="E2:E2000">
-      <formula1>Listas!$O$2:$O$500</formula1>
+      <formula1>Listas!$P$2:$P$500</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3800,43 +3868,43 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>27</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J1" s="20" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L1" s="20" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>34</v>
@@ -3845,10 +3913,10 @@
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D2" s="11">
         <v>46307</v>
@@ -3857,13 +3925,13 @@
         <v>0.8194444444444444</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="21">
@@ -3876,14 +3944,14 @@
         <v>0.8541666666666666</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Tipo" error="Elija un valor de la lista desplegable." sqref="C2:C2000">
-      <formula1>Listas!$T$2:$T$500</formula1>
+      <formula1>Listas!$U$2:$U$500</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha del reporte" error="Escriba una fecha válida (día/mes/año)." sqref="D2:D2000">
       <formula1>21916</formula1>
@@ -3894,7 +3962,7 @@
       <formula2>0.99999</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Técnico" error="Elija un valor de la lista desplegable." sqref="I2:I2000">
-      <formula1>Listas!$R$2:$R$500</formula1>
+      <formula1>Listas!$S$2:$S$500</formula1>
     </dataValidation>
     <dataValidation type="time" allowBlank="1" showErrorMessage="1" errorTitle="Hora de llegada" error="Escriba una hora en formato 24 horas (07:30)." sqref="J2:J2000">
       <formula1>0</formula1>

</xml_diff>